<commit_message>
docs: ajoute le template d'import objectifs à évaluer, MAJ historique
Ajoute template_objectifs_a_evaluer(.xlsx/_exemple.xlsx) pour
/api/interviews/import_objectifs_a_evaluer/ (Matricule, Définition,
Thème, Date de réalisation).

Met à jour la description de la colonne Type Entretien du template
historique : elle est désormais obligatoire, le sélecteur de type par
défaut ayant été retiré de l'interface.
</commit_message>
<xml_diff>
--- a/doc/Exemple Importation/template_entretiens_historique_exemple.xlsx
+++ b/doc/Exemple Importation/template_entretiens_historique_exemple.xlsx
@@ -462,7 +462,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Remplacez la/les ligne(s) d'exemple par vos données. La ligne d'explications (ligne 4) est indicative, à supprimer avant l'import. Le type d'entretien peut être renseigné par ligne (colonne Type Entretien) ou choisi une fois pour tout le fichier au moment de l'import si la colonne est vide.</t>
+          <t>Remplacez la/les ligne(s) d'exemple par vos données. La ligne d'explications (ligne 4) est indicative, à supprimer avant l'import.</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Entretien d'évaluation / Entretien professionnel / Entretien de bilan / Entretien forfait jours et charges / Entretien de fin de carrière (optionnel, sinon reprend le type choisi au moment de l'import)</t>
+          <t>Entretien d'évaluation / Entretien professionnel / Entretien de bilan / Entretien forfait jours et charges / Entretien de fin de carrière (obligatoire)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: corrige le template historique — Type Entretien manquant en ligne 2
La 2e ligne d'exemple avait un Type Entretien vide, alors que la
colonne est désormais obligatoire (plus de type par défaut choisi
dans l'interface) — cette ligne aurait été rejetée à l'import.
</commit_message>
<xml_diff>
--- a/doc/Exemple Importation/template_entretiens_historique_exemple.xlsx
+++ b/doc/Exemple Importation/template_entretiens_historique_exemple.xlsx
@@ -568,6 +568,11 @@
           <t>05/09/2024</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Entretien professionnel</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>

</xml_diff>